<commit_message>
V2.1 Final: Implementation of Quantity-based SO, Procurement Status, and Fixed Reporting Logic
</commit_message>
<xml_diff>
--- a/assets/database.xlsx
+++ b/assets/database.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="25">
   <si>
     <t>No Asset</t>
   </si>
@@ -28,6 +28,9 @@
     <t>Daya</t>
   </si>
   <si>
+    <t>quantity</t>
+  </si>
+  <si>
     <t>Tahun Buat</t>
   </si>
   <si>
@@ -55,31 +58,34 @@
     <t>China</t>
   </si>
   <si>
+    <t>Packing</t>
+  </si>
+  <si>
     <t>80 Ton</t>
   </si>
   <si>
+    <t>Polishing</t>
+  </si>
+  <si>
     <t>100 Ton</t>
   </si>
   <si>
+    <t>Macahine</t>
+  </si>
+  <si>
     <t>150 Ton</t>
   </si>
   <si>
+    <t>Knife</t>
+  </si>
+  <si>
     <t>160 Ton</t>
   </si>
   <si>
-    <t>Packing</t>
-  </si>
-  <si>
-    <t>Polishing</t>
-  </si>
-  <si>
-    <t>Macahine</t>
-  </si>
-  <si>
-    <t>Knife</t>
-  </si>
-  <si>
     <t>Grinding</t>
+  </si>
+  <si>
+    <t>Machining</t>
   </si>
 </sst>
 </file>
@@ -139,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -148,10 +154,13 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="14" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="14" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -374,13 +383,13 @@
     <col customWidth="1" min="3" max="3" width="18.38"/>
     <col customWidth="1" min="4" max="4" width="16.0"/>
     <col customWidth="1" min="5" max="5" width="9.88"/>
-    <col customWidth="1" min="6" max="6" width="15.63"/>
-    <col customWidth="1" min="7" max="7" width="10.25"/>
-    <col customWidth="1" min="8" max="8" width="11.75"/>
-    <col customWidth="1" min="9" max="9" width="10.25"/>
-    <col customWidth="1" min="10" max="10" width="6.13"/>
-    <col customWidth="1" min="11" max="11" width="7.88"/>
-    <col customWidth="1" min="12" max="25" width="8.63"/>
+    <col customWidth="1" min="6" max="7" width="15.63"/>
+    <col customWidth="1" min="8" max="8" width="10.25"/>
+    <col customWidth="1" min="9" max="9" width="11.75"/>
+    <col customWidth="1" min="10" max="10" width="10.25"/>
+    <col customWidth="1" min="11" max="11" width="6.13"/>
+    <col customWidth="1" min="12" max="12" width="7.88"/>
+    <col customWidth="1" min="13" max="26" width="8.63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -399,7 +408,7 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -416,173 +425,316 @@
       </c>
       <c r="K1" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="3">
         <v>15.0</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
+      <c r="F2" s="4">
+        <v>20.0</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
       <c r="B3" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>13</v>
       </c>
       <c r="E3" s="3">
         <v>15.0</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
+      <c r="F3" s="4">
+        <v>15.0</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="3">
         <v>15.0</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="F4" s="4">
+        <v>17.0</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="3">
         <v>15.0</v>
       </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
+      <c r="F5" s="4">
+        <v>20.0</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" s="3">
         <v>15.0</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="F6" s="4">
+        <v>56.0</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="s">
-        <v>11</v>
+      <c r="B7" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" s="3">
         <v>15.0</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>18</v>
-      </c>
+      <c r="F7" s="5">
+        <v>12.0</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
     </row>
     <row r="8">
-      <c r="B8" s="3" t="s">
-        <v>11</v>
+      <c r="B8" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>13</v>
       </c>
       <c r="E8" s="3">
         <v>15.0</v>
       </c>
-      <c r="H8" s="5" t="s">
-        <v>19</v>
+      <c r="F8" s="5">
+        <v>20.0</v>
+      </c>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="3" t="s">
-        <v>11</v>
+      <c r="B9" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="3">
         <v>15.0</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>20</v>
+      <c r="F9" s="5">
+        <v>5.0</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="3" t="s">
-        <v>11</v>
+      <c r="B10" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E10" s="3">
         <v>15.0</v>
       </c>
-      <c r="H10" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="F10" s="5">
+        <v>8.0</v>
+      </c>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="s">
-        <v>11</v>
+      <c r="B11" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" s="3">
         <v>15.0</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="F11" s="5">
+        <v>9.0</v>
+      </c>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="F13" s="4">
+        <v>31.0</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>25.0</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="F15" s="4">
+        <v>15.0</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="B16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>22</v>
       </c>
+      <c r="D16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="F16" s="4">
+        <v>28.0</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>23</v>
+      </c>
     </row>
+    <row r="17" ht="15.75" customHeight="1"/>
+    <row r="18" ht="15.75" customHeight="1"/>
+    <row r="19" ht="15.75" customHeight="1"/>
+    <row r="20" ht="15.75" customHeight="1"/>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
@@ -1558,11 +1710,6 @@
     <row r="993" ht="15.75" customHeight="1"/>
     <row r="994" ht="15.75" customHeight="1"/>
     <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>